<commit_message>
removed subs that left the contract
</commit_message>
<xml_diff>
--- a/sbs_tef.xlsx
+++ b/sbs_tef.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kcollins17\Desktop\github\chc-site\content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slmooradian\git_repos\chc-cfo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C5D31E-4D5F-437E-A724-9C9BC550EDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53CF8EC-33A7-42E1-9FBB-4C8E1FA7C3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3864" yWindow="0" windowWidth="14832" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>Community Action Agency of Butte County, Inc.</t>
   </si>
@@ -71,9 +71,6 @@
     <t>College of the Siskiyous</t>
   </si>
   <si>
-    <t>CSU, East Bay Foundation Inc.</t>
-  </si>
-  <si>
     <t>CSU, Northridge, The University Corporation </t>
   </si>
   <si>
@@ -173,9 +170,6 @@
     <t>CoS</t>
   </si>
   <si>
-    <t>CSUEB</t>
-  </si>
-  <si>
     <t>CSUN</t>
   </si>
   <si>
@@ -294,12 +288,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sonoma State University </t>
-  </si>
-  <si>
-    <t>The Regents of the University of California, Berkeley</t>
-  </si>
-  <si>
-    <t>UCB</t>
   </si>
   <si>
     <t xml:space="preserve">The Regents of the University of California, Davis </t>
@@ -746,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="59.109375" customWidth="1"/>
@@ -755,18 +743,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -774,71 +762,71 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -846,7 +834,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -854,31 +842,31 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -886,7 +874,7 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -894,23 +882,23 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -918,20 +906,20 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B22" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B23" t="s">
         <v>40</v>
@@ -939,34 +927,34 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>98</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -974,7 +962,7 @@
         <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -982,7 +970,7 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -990,15 +978,15 @@
         <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -1019,18 +1007,18 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
@@ -1038,151 +1026,135 @@
         <v>75</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>76</v>
+      </c>
+      <c r="B37" t="s">
         <v>77</v>
-      </c>
-      <c r="B37" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="B40" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="B48" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>86</v>
+        <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B52" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>17</v>
-      </c>
-      <c r="B54" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated sbs_tef with new FFY 27 subs
</commit_message>
<xml_diff>
--- a/sbs_tef.xlsx
+++ b/sbs_tef.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slmooradian\git_repos\chc-cfo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53CF8EC-33A7-42E1-9FBB-4C8E1FA7C3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617FBEE9-1E69-4013-842F-679ACB73B93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="672" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>Community Action Agency of Butte County, Inc.</t>
   </si>
@@ -363,6 +363,138 @@
   </si>
   <si>
     <t>Entity</t>
+  </si>
+  <si>
+    <t>Adventist Health System West (dba Adventist Health)</t>
+  </si>
+  <si>
+    <t>CommonSpirit Health</t>
+  </si>
+  <si>
+    <t>Enloe Medical Center</t>
+  </si>
+  <si>
+    <t>Jordan Crossing Ministries</t>
+  </si>
+  <si>
+    <t>Oroville Rescue Mission</t>
+  </si>
+  <si>
+    <t>Youth for Change</t>
+  </si>
+  <si>
+    <t>Butte County Office of Education</t>
+  </si>
+  <si>
+    <t>Trinity County Office of Education</t>
+  </si>
+  <si>
+    <t>Legal Services of Northern CA</t>
+  </si>
+  <si>
+    <t>Empower Tehama</t>
+  </si>
+  <si>
+    <t>Coast Community College District - Coastline Community College</t>
+  </si>
+  <si>
+    <t>Reedley College</t>
+  </si>
+  <si>
+    <t>Yuba Community College District - Woodland Community College</t>
+  </si>
+  <si>
+    <t>CA Dept of Corrections (Northern CA region)</t>
+  </si>
+  <si>
+    <t>Trinity County Food Assistance</t>
+  </si>
+  <si>
+    <t>Safe Space Winter Shelter, Inc.</t>
+  </si>
+  <si>
+    <t>Home &amp; Heart</t>
+  </si>
+  <si>
+    <t>San Diego Community College District (San Diego Mesa College)</t>
+  </si>
+  <si>
+    <t>Kern Community College District on behalf of Bakersfield College</t>
+  </si>
+  <si>
+    <t>Citrus Community College District</t>
+  </si>
+  <si>
+    <t>Redwoods Community College District - College of the Redwoods</t>
+  </si>
+  <si>
+    <t>CSU Bakersfield Auxiliary for Sponsored Programs Administration</t>
+  </si>
+  <si>
+    <t>WCC</t>
+  </si>
+  <si>
+    <t>CDCR</t>
+  </si>
+  <si>
+    <t>AHSW</t>
+  </si>
+  <si>
+    <t>CSH</t>
+  </si>
+  <si>
+    <t>ENLOE</t>
+  </si>
+  <si>
+    <t>TCFA</t>
+  </si>
+  <si>
+    <t>JCM</t>
+  </si>
+  <si>
+    <t>ORM</t>
+  </si>
+  <si>
+    <t>SSWS</t>
+  </si>
+  <si>
+    <t>Y4C</t>
+  </si>
+  <si>
+    <t>HH</t>
+  </si>
+  <si>
+    <t>BCOE</t>
+  </si>
+  <si>
+    <t>TCOE</t>
+  </si>
+  <si>
+    <t>LSNC</t>
+  </si>
+  <si>
+    <t>ET</t>
+  </si>
+  <si>
+    <t>SDMC</t>
+  </si>
+  <si>
+    <t>BFC</t>
+  </si>
+  <si>
+    <t>CLCC</t>
+  </si>
+  <si>
+    <t>CITRUS</t>
+  </si>
+  <si>
+    <t>CoR</t>
+  </si>
+  <si>
+    <t>CSUB</t>
+  </si>
+  <si>
+    <t>RCC</t>
   </si>
 </sst>
 </file>
@@ -404,8 +536,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -734,14 +869,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B74"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.109375" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>103</v>
       </c>
@@ -749,7 +884,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -757,7 +892,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -765,7 +900,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -773,7 +908,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -781,7 +916,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -789,7 +924,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -797,7 +932,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -805,7 +940,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -813,7 +948,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -821,7 +956,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>60</v>
       </c>
@@ -829,7 +964,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -837,7 +972,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -845,7 +980,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -853,7 +988,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -861,7 +996,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>63</v>
       </c>
@@ -869,7 +1004,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -877,7 +1012,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -885,7 +1020,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -893,7 +1028,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>89</v>
       </c>
@@ -901,7 +1036,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -909,7 +1044,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>91</v>
       </c>
@@ -917,7 +1052,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -925,7 +1060,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>99</v>
       </c>
@@ -933,7 +1068,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -941,7 +1076,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>93</v>
       </c>
@@ -949,7 +1084,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -957,7 +1092,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -965,7 +1100,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>10</v>
       </c>
@@ -973,7 +1108,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -981,7 +1116,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -989,7 +1124,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>69</v>
       </c>
@@ -997,7 +1132,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>71</v>
       </c>
@@ -1005,7 +1140,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -1013,7 +1148,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>73</v>
       </c>
@@ -1021,7 +1156,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -1029,7 +1164,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>76</v>
       </c>
@@ -1037,7 +1172,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>97</v>
       </c>
@@ -1045,7 +1180,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -1053,7 +1188,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>101</v>
       </c>
@@ -1061,7 +1196,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>79</v>
       </c>
@@ -1069,7 +1204,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -1077,7 +1212,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -1085,7 +1220,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>80</v>
       </c>
@@ -1093,7 +1228,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>17</v>
       </c>
@@ -1101,7 +1236,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>23</v>
       </c>
@@ -1109,7 +1244,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
@@ -1117,7 +1252,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -1125,7 +1260,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -1133,7 +1268,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -1141,7 +1276,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -1149,17 +1284,194 @@
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>16</v>
       </c>
       <c r="B52" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>116</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>117</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>105</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>106</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>107</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>108</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>119</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>109</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>111</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>112</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>113</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>122</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>114</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>123</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>124</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>125</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>115</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>